<commit_message>
update version + path fa8a4759d7c8bbfecec8abdc99238d20fe48c43a
</commit_message>
<xml_diff>
--- a/IG_LGC_config/ig/CodeSystem-competence-code-system.xlsx
+++ b/IG_LGC_config/ig/CodeSystem-competence-code-system.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>0.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T09:57:24+00:00</t>
+    <t>2026-06-25T10:01:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>